<commit_message>
fix: correct Gantt phases for DEV1-DEV5 and the H1 dependency
Task List sheet: the five development work packages (DEV1-DEV5) were labelled
Design; they are Development. H1 (GitHub maintenance) declared a dependency on
DEV1 but started two days before DEV1 finished; it now depends on D3, which
delivers the README and directory structure it actually needs.
</commit_message>
<xml_diff>
--- a/docs/original/04_Project_Gantt_Chart.xlsx
+++ b/docs/original/04_Project_Gantt_Chart.xlsx
@@ -2039,7 +2039,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="I21" s="7" t="n"/>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Development</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3530,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Development</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Development</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Development</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Development</t>
         </is>
       </c>
     </row>
@@ -3840,7 +3840,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>DEV1</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">

</xml_diff>